<commit_message>
fix: dashboard debug and react test
</commit_message>
<xml_diff>
--- a/ShipSafe_Tasks.xlsx
+++ b/ShipSafe_Tasks.xlsx
@@ -558,7 +558,11 @@
           <t>frontend/package.json</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr"/>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Manifest known-CVE artifact</t>
@@ -576,7 +580,7 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
final: README + Excel + bob_sessions
</commit_message>
<xml_diff>
--- a/ShipSafe_Tasks.xlsx
+++ b/ShipSafe_Tasks.xlsx
@@ -587,7 +587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q18"/>
+  <dimension ref="A1:R18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -607,6 +607,7 @@
     <col width="46" customWidth="1" min="15" max="15"/>
     <col width="10" customWidth="1" min="16" max="16"/>
     <col width="52" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -622,7 +623,7 @@
       </c>
       <c r="C1" s="8" t="inlineStr">
         <is>
-          <t>Run: 2026-08-29 19:17</t>
+          <t>Run: 2026-08-29 19:45</t>
         </is>
       </c>
       <c r="D1" s="9" t="inlineStr">
@@ -635,7 +636,11 @@
           <t>Verdict: 🔴 NO-GO — see findings below</t>
         </is>
       </c>
-      <c r="F1" s="10" t="n"/>
+      <c r="F1" s="8" t="inlineStr">
+        <is>
+          <t>No PR</t>
+        </is>
+      </c>
       <c r="G1" s="10" t="n"/>
       <c r="H1" s="10" t="n"/>
       <c r="I1" s="10" t="n"/>
@@ -646,7 +651,8 @@
       <c r="N1" s="10" t="n"/>
       <c r="O1" s="10" t="n"/>
       <c r="P1" s="10" t="n"/>
-      <c r="Q1" s="11">
+      <c r="Q1" s="10" t="n"/>
+      <c r="R1" s="11">
         <f>HYPERLINK("http://127.0.0.1:5001","Dashboard")</f>
         <v/>
       </c>
@@ -737,6 +743,11 @@
           <t>Created From Why</t>
         </is>
       </c>
+      <c r="R2" s="12" t="inlineStr">
+        <is>
+          <t>PR Link</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
@@ -772,7 +783,7 @@
       </c>
       <c r="H3" s="13" t="inlineStr">
         <is>
-          <t>2026-08-29 19:17</t>
+          <t>2026-08-29 19:45</t>
         </is>
       </c>
       <c r="I3" s="13" t="inlineStr">
@@ -796,7 +807,7 @@
       </c>
       <c r="M3" s="13" t="inlineStr">
         <is>
-          <t>2026-08-29 19:17</t>
+          <t>2026-08-29 19:45</t>
         </is>
       </c>
       <c r="N3" s="13" t="inlineStr">
@@ -819,6 +830,7 @@
           <t>API compatibility gate — prevents breaking changes reaching production consumers</t>
         </is>
       </c>
+      <c r="R3" s="14" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="15" t="inlineStr">
@@ -854,12 +866,12 @@
       </c>
       <c r="H4" s="15" t="inlineStr">
         <is>
-          <t>2026-08-29 19:17</t>
+          <t>2026-08-29 19:45</t>
         </is>
       </c>
       <c r="I4" s="15" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-29 17:00</t>
         </is>
       </c>
       <c r="J4" s="14">
@@ -901,6 +913,7 @@
           <t>Supply-chain security — known CVE in a direct dependency blocks safe deployment</t>
         </is>
       </c>
+      <c r="R4" s="14" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="13" t="inlineStr">
@@ -936,7 +949,7 @@
       </c>
       <c r="H5" s="13" t="inlineStr">
         <is>
-          <t>2026-08-29 19:17</t>
+          <t>2026-08-29 19:45</t>
         </is>
       </c>
       <c r="I5" s="13" t="inlineStr">
@@ -960,7 +973,7 @@
       </c>
       <c r="M5" s="13" t="inlineStr">
         <is>
-          <t>2026-08-29 19:17</t>
+          <t>2026-08-29 19:45</t>
         </is>
       </c>
       <c r="N5" s="13" t="inlineStr">
@@ -983,6 +996,7 @@
           <t>Python dependency audit — CVE in requirements.txt or lockfile poses runtime risk</t>
         </is>
       </c>
+      <c r="R5" s="14" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="15" t="inlineStr">
@@ -1022,12 +1036,12 @@
       </c>
       <c r="H6" s="15" t="inlineStr">
         <is>
-          <t>2026-08-29 19:17</t>
+          <t>2026-08-29 19:45</t>
         </is>
       </c>
       <c r="I6" s="15" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-29 17:00</t>
         </is>
       </c>
       <c r="J6" s="14">
@@ -1069,6 +1083,7 @@
           <t>Secrets management — VAULT_ID must be bound before the app can reach the vault</t>
         </is>
       </c>
+      <c r="R6" s="14" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
@@ -1104,12 +1119,12 @@
       </c>
       <c r="H7" s="15" t="inlineStr">
         <is>
-          <t>2026-08-29 19:17</t>
+          <t>2026-08-29 19:45</t>
         </is>
       </c>
       <c r="I7" s="15" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-29 17:00</t>
         </is>
       </c>
       <c r="J7" s="14">
@@ -1151,6 +1166,7 @@
           <t>Credential hygiene — hardcoded secrets in config files leak via version control</t>
         </is>
       </c>
+      <c r="R7" s="14" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="13" t="inlineStr">
@@ -1190,7 +1206,7 @@
       </c>
       <c r="H8" s="13" t="inlineStr">
         <is>
-          <t>2026-08-29 19:17</t>
+          <t>2026-08-29 19:45</t>
         </is>
       </c>
       <c r="I8" s="13" t="inlineStr">
@@ -1237,6 +1253,7 @@
           <t>Attack surface — wildcard actuator exposure allows unauthenticated admin access</t>
         </is>
       </c>
+      <c r="R8" s="14" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="13" t="inlineStr">
@@ -1272,7 +1289,7 @@
       </c>
       <c r="H9" s="13" t="inlineStr">
         <is>
-          <t>2026-08-29 19:17</t>
+          <t>2026-08-29 19:45</t>
         </is>
       </c>
       <c r="I9" s="13" t="inlineStr">
@@ -1319,6 +1336,7 @@
           <t>Transport security — plain HTTP in production exposes credentials and data in transit</t>
         </is>
       </c>
+      <c r="R9" s="14" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="13" t="inlineStr">
@@ -1354,7 +1372,7 @@
       </c>
       <c r="H10" s="13" t="inlineStr">
         <is>
-          <t>2026-08-29 19:17</t>
+          <t>2026-08-29 19:45</t>
         </is>
       </c>
       <c r="I10" s="13" t="inlineStr">
@@ -1401,6 +1419,7 @@
           <t>Authentication gate — no security dependency means all endpoints are unprotected</t>
         </is>
       </c>
+      <c r="R10" s="14" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="17" t="inlineStr">
@@ -1436,10 +1455,14 @@
       </c>
       <c r="H11" s="17" t="inlineStr">
         <is>
-          <t>2026-08-29 19:17</t>
-        </is>
-      </c>
-      <c r="I11" s="17" t="inlineStr"/>
+          <t>2026-08-29 19:45</t>
+        </is>
+      </c>
+      <c r="I11" s="17" t="inlineStr">
+        <is>
+          <t>2026-09-04 17:00</t>
+        </is>
+      </c>
       <c r="J11" s="14">
         <f>HYPERLINK("file:////Users/cerinrosechelladurai/Desktop/shipsafe-release-guardian/src/pom.xml", "Open")</f>
         <v/>
@@ -1479,6 +1502,7 @@
           <t>Data integrity — unmanaged schema changes risk migration failures on deploy</t>
         </is>
       </c>
+      <c r="R11" s="14" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="17" t="inlineStr">
@@ -1514,10 +1538,14 @@
       </c>
       <c r="H12" s="17" t="inlineStr">
         <is>
-          <t>2026-08-29 19:17</t>
-        </is>
-      </c>
-      <c r="I12" s="17" t="inlineStr"/>
+          <t>2026-08-29 19:45</t>
+        </is>
+      </c>
+      <c r="I12" s="17" t="inlineStr">
+        <is>
+          <t>2026-09-04 17:00</t>
+        </is>
+      </c>
       <c r="J12" s="14">
         <f>HYPERLINK("file:////Users/cerinrosechelladurai/Desktop/shipsafe-release-guardian/src/Dockerfile", "Open")</f>
         <v/>
@@ -1534,7 +1562,7 @@
       </c>
       <c r="M12" s="17" t="inlineStr">
         <is>
-          <t>2026-08-29 19:17</t>
+          <t>2026-08-29 19:45</t>
         </is>
       </c>
       <c r="N12" s="17" t="inlineStr">
@@ -1557,6 +1585,7 @@
           <t>Container hygiene — ports below 1024 require root privileges in the container</t>
         </is>
       </c>
+      <c r="R12" s="14" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="13" t="inlineStr">
@@ -1592,7 +1621,7 @@
       </c>
       <c r="H13" s="13" t="inlineStr">
         <is>
-          <t>2026-08-29 19:17</t>
+          <t>2026-08-29 19:45</t>
         </is>
       </c>
       <c r="I13" s="13" t="inlineStr">
@@ -1616,7 +1645,7 @@
       </c>
       <c r="M13" s="13" t="inlineStr">
         <is>
-          <t>2026-08-29 19:17</t>
+          <t>2026-08-29 19:45</t>
         </is>
       </c>
       <c r="N13" s="13" t="inlineStr">
@@ -1639,6 +1668,7 @@
           <t>Infrastructure hygiene — hardcoded S3 bucket couples pipeline to a specific account</t>
         </is>
       </c>
+      <c r="R13" s="14" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="17" t="inlineStr">
@@ -1674,10 +1704,14 @@
       </c>
       <c r="H14" s="17" t="inlineStr">
         <is>
-          <t>2026-08-29 19:17</t>
-        </is>
-      </c>
-      <c r="I14" s="17" t="inlineStr"/>
+          <t>2026-08-29 19:45</t>
+        </is>
+      </c>
+      <c r="I14" s="17" t="inlineStr">
+        <is>
+          <t>2026-09-04 17:00</t>
+        </is>
+      </c>
       <c r="J14" s="14">
         <f>HYPERLINK("file:////Users/cerinrosechelladurai/Desktop/shipsafe-release-guardian/notebook.ipynb", "Open")</f>
         <v/>
@@ -1694,7 +1728,7 @@
       </c>
       <c r="M14" s="17" t="inlineStr">
         <is>
-          <t>2026-08-29 19:17</t>
+          <t>2026-08-29 19:45</t>
         </is>
       </c>
       <c r="N14" s="17" t="inlineStr">
@@ -1717,6 +1751,7 @@
           <t>Notebook security — api_key literals in notebooks leak credentials via git history</t>
         </is>
       </c>
+      <c r="R14" s="14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="18" t="inlineStr">
@@ -1752,7 +1787,7 @@
       </c>
       <c r="H15" s="18" t="inlineStr">
         <is>
-          <t>2026-08-29 19:17</t>
+          <t>2026-08-29 19:45</t>
         </is>
       </c>
       <c r="I15" s="18" t="inlineStr"/>
@@ -1772,7 +1807,7 @@
       </c>
       <c r="M15" s="18" t="inlineStr">
         <is>
-          <t>2026-08-29 19:17</t>
+          <t>2026-08-29 19:45</t>
         </is>
       </c>
       <c r="N15" s="18" t="inlineStr">
@@ -1795,6 +1830,7 @@
           <t>Notebook portability — hardcoded local paths break notebook execution in CI/CD</t>
         </is>
       </c>
+      <c r="R15" s="14" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="18" t="inlineStr">
@@ -1830,7 +1866,7 @@
       </c>
       <c r="H16" s="18" t="inlineStr">
         <is>
-          <t>2026-08-29 19:17</t>
+          <t>2026-08-29 19:45</t>
         </is>
       </c>
       <c r="I16" s="18" t="inlineStr"/>
@@ -1850,7 +1886,7 @@
       </c>
       <c r="M16" s="18" t="inlineStr">
         <is>
-          <t>2026-08-29 19:17</t>
+          <t>2026-08-29 19:45</t>
         </is>
       </c>
       <c r="N16" s="18" t="inlineStr">
@@ -1873,6 +1909,7 @@
           <t>ML reproducibility — missing CUDA env var causes silent CPU fallback on GPU nodes</t>
         </is>
       </c>
+      <c r="R16" s="14" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="15" t="inlineStr">
@@ -1908,12 +1945,12 @@
       </c>
       <c r="H17" s="15" t="inlineStr">
         <is>
-          <t>2026-08-29 19:17</t>
+          <t>2026-08-29 19:45</t>
         </is>
       </c>
       <c r="I17" s="15" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-29 17:00</t>
         </is>
       </c>
       <c r="J17" s="14">
@@ -1955,6 +1992,7 @@
           <t>Deploy-time secrets — VAULT_ID absent in codeengine.yaml means app cannot start</t>
         </is>
       </c>
+      <c r="R17" s="14" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="15" t="inlineStr">
@@ -1994,12 +2032,12 @@
       </c>
       <c r="H18" s="15" t="inlineStr">
         <is>
-          <t>2026-08-29 19:17</t>
+          <t>2026-08-29 19:45</t>
         </is>
       </c>
       <c r="I18" s="15" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-29 17:00</t>
         </is>
       </c>
       <c r="J18" s="14">
@@ -2041,6 +2079,7 @@
           <t>Dependency hygiene — phantom artifact fails resolution and blocks the build</t>
         </is>
       </c>
+      <c r="R18" s="14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2053,7 +2092,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2216,6 +2255,102 @@
         <v>16</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-29 19:37</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>🔴 NO-GO — see findings below</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>9</v>
+      </c>
+      <c r="D7" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-29 19:37</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>🔴 NO-GO — see findings below</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>9</v>
+      </c>
+      <c r="D8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-29 19:37</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>🔴 NO-GO — see findings below</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>9</v>
+      </c>
+      <c r="D9" t="n">
+        <v>5</v>
+      </c>
+      <c r="E9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F9" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-29 19:45</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>🔴 NO-GO — see findings below</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>9</v>
+      </c>
+      <c r="D10" t="n">
+        <v>5</v>
+      </c>
+      <c r="E10" t="n">
+        <v>2</v>
+      </c>
+      <c r="F10" t="n">
+        <v>16</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>